<commit_message>
Emergency: Manual data sync for research fields and reset V8.9.9.5
</commit_message>
<xml_diff>
--- a/data/trending_integrated.xlsx
+++ b/data/trending_integrated.xlsx
@@ -508,25 +508,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>옵티시스</t>
+          <t>캡스톤파트너스</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>16120</v>
+        <v>4645</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>+30.00%</t>
+          <t>+29.93%</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>-0.31</v>
+        <v>-3.53</v>
       </c>
       <c r="E2" t="n">
-        <v>136</v>
+        <v>173</v>
       </c>
       <c r="F2" t="n">
-        <v>1.13</v>
+        <v>2.95</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -534,10 +534,10 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>12400</v>
+        <v>3575</v>
       </c>
       <c r="I2" t="n">
-        <v>1.44</v>
+        <v>6.48</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -557,48 +557,48 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>109080</t>
+          <t>452300</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>109080</t>
+          <t>452300</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>캡스톤파트너스</t>
+          <t>광전자</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4645</v>
+        <v>7520</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>+29.93%</t>
+          <t>+29.88%</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>-3.53</v>
+        <v>-0.28</v>
       </c>
       <c r="E3" t="n">
-        <v>172</v>
+        <v>309</v>
       </c>
       <c r="F3" t="n">
-        <v>2.95</v>
+        <v>18.2</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>KOSDAQ</t>
+          <t>KOSPI</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>3575</v>
+        <v>5790</v>
       </c>
       <c r="I3" t="n">
-        <v>6.48</v>
+        <v>18.48</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -618,48 +618,48 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>452300</t>
+          <t>017900</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>452300</t>
+          <t>017900</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>광전자</t>
+          <t>아크릴</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7520</v>
+        <v>37650</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>+29.88%</t>
+          <t>+19.33%</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>-0.28</v>
+        <v>-1.12</v>
       </c>
       <c r="E4" t="n">
-        <v>304</v>
+        <v>272</v>
       </c>
       <c r="F4" t="n">
-        <v>18.2</v>
+        <v>3.71</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>KOSPI</t>
+          <t>KOSDAQ</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>5790</v>
+        <v>31550</v>
       </c>
       <c r="I4" t="n">
-        <v>18.48</v>
+        <v>4.83</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -679,37 +679,37 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>017900</t>
+          <t>0007C0</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>017900</t>
+          <t>0007C0</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>아크릴</t>
+          <t>프로이천</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>37650</v>
+        <v>2900</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>+19.33%</t>
+          <t>+18.37%</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>-1.12</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>271</v>
+        <v>261</v>
       </c>
       <c r="F5" t="n">
-        <v>3.71</v>
+        <v>1.92</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -717,10 +717,10 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>31550</v>
+        <v>2450</v>
       </c>
       <c r="I5" t="n">
-        <v>4.83</v>
+        <v>0.92</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -740,37 +740,37 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>0007C0</t>
+          <t>321260</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>0007C0</t>
+          <t>321260</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>프로이천</t>
+          <t>서울반도체</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2900</v>
+        <v>10300</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>+18.37%</t>
+          <t>+17.58%</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>-0.83</v>
       </c>
       <c r="E6" t="n">
-        <v>261</v>
+        <v>152</v>
       </c>
       <c r="F6" t="n">
-        <v>1.92</v>
+        <v>7.85</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -778,10 +778,10 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>2450</v>
+        <v>8760</v>
       </c>
       <c r="I6" t="n">
-        <v>0.92</v>
+        <v>8.68</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -801,48 +801,48 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>321260</t>
+          <t>046890</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>321260</t>
+          <t>046890</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>서울반도체</t>
+          <t>풍산홀딩스</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>10300</v>
+        <v>54800</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>+17.58%</t>
+          <t>+15.98%</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>-0.83</v>
+        <v>-1.21</v>
       </c>
       <c r="E7" t="n">
-        <v>152</v>
+        <v>786</v>
       </c>
       <c r="F7" t="n">
-        <v>7.85</v>
+        <v>11.62</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>KOSDAQ</t>
+          <t>KOSPI</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>8760</v>
+        <v>47250</v>
       </c>
       <c r="I7" t="n">
-        <v>8.68</v>
+        <v>12.83</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -862,48 +862,48 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>046890</t>
+          <t>005810</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>046890</t>
+          <t>005810</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>풍산홀딩스</t>
+          <t>창해에탄올</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>54800</v>
+        <v>12010</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>+15.98%</t>
+          <t>+15.93%</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>-1.21</v>
+        <v>-0.54</v>
       </c>
       <c r="E8" t="n">
-        <v>782</v>
+        <v>572</v>
       </c>
       <c r="F8" t="n">
-        <v>11.62</v>
+        <v>1.37</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>KOSPI</t>
+          <t>KOSDAQ</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>47250</v>
+        <v>10360</v>
       </c>
       <c r="I8" t="n">
-        <v>12.83</v>
+        <v>1.91</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -923,37 +923,37 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>005810</t>
+          <t>004650</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>005810</t>
+          <t>004650</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>창해에탄올</t>
+          <t>리센스메디컬</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>12010</v>
+        <v>23600</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>+15.93%</t>
+          <t>+12.38%</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>-0.54</v>
+        <v>0.74</v>
       </c>
       <c r="E9" t="n">
-        <v>569</v>
+        <v>246</v>
       </c>
       <c r="F9" t="n">
-        <v>1.37</v>
+        <v>1.91</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -961,10 +961,10 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>10360</v>
+        <v>21000</v>
       </c>
       <c r="I9" t="n">
-        <v>1.91</v>
+        <v>1.17</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -984,37 +984,37 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>004650</t>
+          <t>394420</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>004650</t>
+          <t>394420</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>리센스메디컬</t>
+          <t>흥구석유</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>23600</v>
+        <v>22850</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>+12.38%</t>
+          <t>+9.86%</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.74</v>
+        <v>1.11</v>
       </c>
       <c r="E10" t="n">
-        <v>246</v>
+        <v>1017</v>
       </c>
       <c r="F10" t="n">
-        <v>1.91</v>
+        <v>1.22</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1022,10 +1022,10 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>21000</v>
+        <v>20800</v>
       </c>
       <c r="I10" t="n">
-        <v>1.17</v>
+        <v>0.11</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -1045,48 +1045,48 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>394420</t>
+          <t>024060</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>394420</t>
+          <t>024060</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>흥구석유</t>
+          <t>엘앤에프</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>22850</v>
+        <v>185000</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>+9.86%</t>
+          <t>+8.44%</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1.11</v>
+        <v>0.45</v>
       </c>
       <c r="E11" t="n">
-        <v>993</v>
+        <v>286</v>
       </c>
       <c r="F11" t="n">
-        <v>1.22</v>
+        <v>19.75</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>KOSDAQ</t>
+          <t>KOSPI</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>20800</v>
+        <v>170600</v>
       </c>
       <c r="I11" t="n">
-        <v>0.11</v>
+        <v>19.3</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -1106,48 +1106,48 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>024060</t>
+          <t>066970</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>024060</t>
+          <t>066970</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>엘앤에프</t>
+          <t>파워넷</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>185000</v>
+        <v>5680</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>+8.44%</t>
+          <t>+8.19%</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.45</v>
+        <v>-1.94</v>
       </c>
       <c r="E12" t="n">
-        <v>283</v>
+        <v>191</v>
       </c>
       <c r="F12" t="n">
-        <v>19.75</v>
+        <v>2.48</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>KOSPI</t>
+          <t>KOSDAQ</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>170600</v>
+        <v>5250</v>
       </c>
       <c r="I12" t="n">
-        <v>19.3</v>
+        <v>4.42</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -1167,48 +1167,48 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>066970</t>
+          <t>037030</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>066970</t>
+          <t>037030</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>파워넷</t>
+          <t>에코프로머티</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>5680</v>
+        <v>73100</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>+8.19%</t>
+          <t>+6.10%</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>-1.94</v>
+        <v>0.11</v>
       </c>
       <c r="E13" t="n">
-        <v>191</v>
+        <v>283</v>
       </c>
       <c r="F13" t="n">
-        <v>2.48</v>
+        <v>16.74</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>KOSDAQ</t>
+          <t>KOSPI</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>5250</v>
+        <v>68900</v>
       </c>
       <c r="I13" t="n">
-        <v>4.42</v>
+        <v>16.63</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -1228,37 +1228,37 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>037030</t>
+          <t>450080</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>037030</t>
+          <t>450080</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>에코프로머티</t>
+          <t>한화에어로스페이스</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>73100</v>
+        <v>1537000</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>+6.10%</t>
+          <t>+6.00%</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.11</v>
+        <v>0.19</v>
       </c>
       <c r="E14" t="n">
-        <v>282</v>
+        <v>133</v>
       </c>
       <c r="F14" t="n">
-        <v>16.74</v>
+        <v>45.38</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1266,10 +1266,10 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>68900</v>
+        <v>1450000</v>
       </c>
       <c r="I14" t="n">
-        <v>16.63</v>
+        <v>45.19</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -1289,48 +1289,48 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>450080</t>
+          <t>012450</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>450080</t>
+          <t>012450</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>한화에어로스페이스</t>
+          <t>풍국주정</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1537000</v>
+        <v>11140</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>+6.00%</t>
+          <t>+5.00%</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.19</v>
+        <v>-0.03</v>
       </c>
       <c r="E15" t="n">
         <v>130</v>
       </c>
       <c r="F15" t="n">
-        <v>45.38</v>
+        <v>0.9</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>KOSPI</t>
+          <t>KOSDAQ</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>1450000</v>
+        <v>10610</v>
       </c>
       <c r="I15" t="n">
-        <v>45.19</v>
+        <v>0.93</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
@@ -1350,48 +1350,48 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>012450</t>
+          <t>023900</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>012450</t>
+          <t>023900</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>풍국주정</t>
+          <t>한국ANKOR유전</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>11140</v>
+        <v>280</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>+5.00%</t>
+          <t>+4.87%</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>-0.03</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="E16" t="n">
-        <v>130</v>
+        <v>147</v>
       </c>
       <c r="F16" t="n">
-        <v>0.9</v>
+        <v>1.8</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>KOSDAQ</t>
+          <t>KOSPI</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>10610</v>
+        <v>267</v>
       </c>
       <c r="I16" t="n">
-        <v>0.93</v>
+        <v>0.86</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -1411,37 +1411,37 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>023900</t>
+          <t>152550</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>023900</t>
+          <t>152550</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>한국ANKOR유전</t>
+          <t>삼성E&amp;A</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>280</v>
+        <v>47800</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>+4.87%</t>
+          <t>+4.71%</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.9399999999999999</v>
+        <v>-0.14</v>
       </c>
       <c r="E17" t="n">
-        <v>146</v>
+        <v>768</v>
       </c>
       <c r="F17" t="n">
-        <v>1.8</v>
+        <v>45.1</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1449,10 +1449,10 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>267</v>
+        <v>45650</v>
       </c>
       <c r="I17" t="n">
-        <v>0.86</v>
+        <v>45.24</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -1472,48 +1472,48 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>152550</t>
+          <t>028050</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>152550</t>
+          <t>028050</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>삼성E&amp;A</t>
+          <t>세림B&amp;G</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>47800</v>
+        <v>2385</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>+4.71%</t>
+          <t>+4.61%</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>-0.14</v>
+        <v>0.41</v>
       </c>
       <c r="E18" t="n">
-        <v>764</v>
+        <v>158</v>
       </c>
       <c r="F18" t="n">
-        <v>45.1</v>
+        <v>2.92</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>KOSPI</t>
+          <t>KOSDAQ</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>45650</v>
+        <v>2280</v>
       </c>
       <c r="I18" t="n">
-        <v>45.24</v>
+        <v>2.51</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -1533,48 +1533,48 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>028050</t>
+          <t>340440</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>028050</t>
+          <t>340440</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>세림B&amp;G</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2385</v>
+        <v>46400</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>+4.61%</t>
+          <t>+3.46%</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.41</v>
+        <v>0.14</v>
       </c>
       <c r="E19" t="n">
-        <v>157</v>
+        <v>172</v>
       </c>
       <c r="F19" t="n">
-        <v>2.92</v>
+        <v>29.58</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>KOSDAQ</t>
+          <t>KOSPI</t>
         </is>
       </c>
       <c r="H19" t="n">
-        <v>2280</v>
+        <v>44850</v>
       </c>
       <c r="I19" t="n">
-        <v>2.51</v>
+        <v>29.44</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
@@ -1594,37 +1594,37 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>340440</t>
+          <t>035720</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>340440</t>
+          <t>035720</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>46400</v>
+        <v>916000</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>+3.46%</t>
+          <t>+3.39%</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.14</v>
+        <v>0.08</v>
       </c>
       <c r="E20" t="n">
-        <v>170</v>
+        <v>1029</v>
       </c>
       <c r="F20" t="n">
-        <v>29.58</v>
+        <v>52.69</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1632,10 +1632,10 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>44850</v>
+        <v>886000</v>
       </c>
       <c r="I20" t="n">
-        <v>29.44</v>
+        <v>52.61</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -1655,37 +1655,37 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>035720</t>
+          <t>000660</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>035720</t>
+          <t>000660</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>한화시스템</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>916000</v>
+        <v>131700</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>+3.39%</t>
+          <t>+3.21%</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.08</v>
+        <v>0.17</v>
       </c>
       <c r="E21" t="n">
-        <v>994</v>
+        <v>451</v>
       </c>
       <c r="F21" t="n">
-        <v>52.69</v>
+        <v>9.01</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1693,10 +1693,10 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>886000</v>
+        <v>127600</v>
       </c>
       <c r="I21" t="n">
-        <v>52.61</v>
+        <v>8.84</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
@@ -1716,37 +1716,37 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>000660</t>
+          <t>272210</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>000660</t>
+          <t>272210</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>한화시스템</t>
+          <t>남선알미늄</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>131700</v>
+        <v>2180</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>+3.21%</t>
+          <t>+2.35%</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.17</v>
+        <v>-0.7</v>
       </c>
       <c r="E22" t="n">
-        <v>446</v>
+        <v>482</v>
       </c>
       <c r="F22" t="n">
-        <v>9.01</v>
+        <v>1.9</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1754,10 +1754,10 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>127600</v>
+        <v>2130</v>
       </c>
       <c r="I22" t="n">
-        <v>8.84</v>
+        <v>2.6</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -1777,37 +1777,37 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>272210</t>
+          <t>008350</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>272210</t>
+          <t>008350</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>남선알미늄</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2180</v>
+        <v>196500</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>+2.35%</t>
+          <t>+1.76%</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>-0.7</v>
+        <v>-0.05</v>
       </c>
       <c r="E23" t="n">
-        <v>476</v>
+        <v>1189</v>
       </c>
       <c r="F23" t="n">
-        <v>1.9</v>
+        <v>48.39</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1815,10 +1815,10 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>2130</v>
+        <v>193100</v>
       </c>
       <c r="I23" t="n">
-        <v>2.6</v>
+        <v>48.44</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -1838,48 +1838,48 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>008350</t>
+          <t>005930</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>008350</t>
+          <t>005930</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>우리로</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>196500</v>
+        <v>7070</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>+1.76%</t>
+          <t>+1.73%</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>-0.05</v>
+        <v>0.54</v>
       </c>
       <c r="E24" t="n">
-        <v>1008</v>
+        <v>313</v>
       </c>
       <c r="F24" t="n">
-        <v>48.39</v>
+        <v>2.82</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>KOSPI</t>
+          <t>KOSDAQ</t>
         </is>
       </c>
       <c r="H24" t="n">
-        <v>193100</v>
+        <v>6950</v>
       </c>
       <c r="I24" t="n">
-        <v>48.44</v>
+        <v>2.28</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
@@ -1899,45 +1899,45 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>005930</t>
+          <t>046970</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>005930</t>
+          <t>046970</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>우리로</t>
+          <t>대영포장</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>7070</v>
+        <v>1288</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>+1.73%</t>
+          <t>+1.42%</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.54</v>
+        <v>-0.93</v>
       </c>
       <c r="E25" t="n">
-        <v>312</v>
+        <v>156</v>
       </c>
       <c r="F25" t="n">
-        <v>2.82</v>
+        <v>1.35</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>KOSDAQ</t>
+          <t>KOSPI</t>
         </is>
       </c>
       <c r="H25" t="n">
-        <v>6950</v>
+        <v>1270</v>
       </c>
       <c r="I25" t="n">
         <v>2.28</v>
@@ -1960,37 +1960,37 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>046970</t>
+          <t>014160</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>046970</t>
+          <t>014160</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>대영포장</t>
+          <t>삼성전자우</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1288</v>
+        <v>130900</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>+1.42%</t>
+          <t>+1.39%</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>-0.93</v>
+        <v>-0.06</v>
       </c>
       <c r="E26" t="n">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="F26" t="n">
-        <v>1.35</v>
+        <v>76.15000000000001</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1998,10 +1998,10 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>1270</v>
+        <v>129100</v>
       </c>
       <c r="I26" t="n">
-        <v>2.28</v>
+        <v>76.20999999999999</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
@@ -2021,48 +2021,48 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>014160</t>
+          <t>005935</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>014160</t>
+          <t>005935</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>삼성전자우</t>
+          <t>기가레인</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>130900</v>
+        <v>2400</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>+1.39%</t>
+          <t>+0.42%</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>-0.06</v>
+        <v>-0.34</v>
       </c>
       <c r="E27" t="n">
-        <v>148</v>
+        <v>200</v>
       </c>
       <c r="F27" t="n">
-        <v>76.15000000000001</v>
+        <v>1.53</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>KOSPI</t>
+          <t>KOSDAQ</t>
         </is>
       </c>
       <c r="H27" t="n">
-        <v>129100</v>
+        <v>2390</v>
       </c>
       <c r="I27" t="n">
-        <v>76.20999999999999</v>
+        <v>1.87</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -2082,48 +2082,48 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>005935</t>
+          <t>049080</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>005935</t>
+          <t>049080</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>기가레인</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>2400</v>
+        <v>17350</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>+0.42%</t>
+          <t>+0.23%</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>-0.34</v>
+        <v>-0.08</v>
       </c>
       <c r="E28" t="n">
-        <v>199</v>
+        <v>339</v>
       </c>
       <c r="F28" t="n">
-        <v>1.53</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>KOSDAQ</t>
+          <t>KOSPI</t>
         </is>
       </c>
       <c r="H28" t="n">
-        <v>2390</v>
+        <v>17310</v>
       </c>
       <c r="I28" t="n">
-        <v>1.87</v>
+        <v>9.630000000000001</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
@@ -2143,37 +2143,37 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>049080</t>
+          <t>047040</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>049080</t>
+          <t>047040</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>대우건설</t>
+          <t>흥아해운</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>17350</v>
+        <v>3795</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>+0.23%</t>
+          <t>+0.13%</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>-0.08</v>
+        <v>0.18</v>
       </c>
       <c r="E29" t="n">
-        <v>336</v>
+        <v>804</v>
       </c>
       <c r="F29" t="n">
-        <v>9.550000000000001</v>
+        <v>1.54</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -2181,10 +2181,10 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>17310</v>
+        <v>3790</v>
       </c>
       <c r="I29" t="n">
-        <v>9.630000000000001</v>
+        <v>1.36</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
@@ -2204,37 +2204,37 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>047040</t>
+          <t>003280</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>047040</t>
+          <t>003280</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>흥아해운</t>
+          <t>후성</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>3795</v>
+        <v>9870</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>+0.13%</t>
+          <t>-0.30%</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.18</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E30" t="n">
-        <v>783</v>
+        <v>201</v>
       </c>
       <c r="F30" t="n">
-        <v>1.54</v>
+        <v>7.18</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -2242,10 +2242,10 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>3790</v>
+        <v>9900</v>
       </c>
       <c r="I30" t="n">
-        <v>1.36</v>
+        <v>6.62</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
@@ -2265,48 +2265,48 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>003280</t>
+          <t>093370</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>003280</t>
+          <t>093370</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>후성</t>
+          <t>에코플라스틱</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>9870</v>
+        <v>4000</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>-0.30%</t>
+          <t>-0.50%</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.5600000000000001</v>
+        <v>-0.76</v>
       </c>
       <c r="E31" t="n">
-        <v>199</v>
+        <v>130</v>
       </c>
       <c r="F31" t="n">
-        <v>7.18</v>
+        <v>0.72</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>KOSPI</t>
+          <t>KOSDAQ</t>
         </is>
       </c>
       <c r="H31" t="n">
-        <v>9900</v>
+        <v>4020</v>
       </c>
       <c r="I31" t="n">
-        <v>6.62</v>
+        <v>1.48</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
@@ -2326,12 +2326,12 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>093370</t>
+          <t>038110</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>093370</t>
+          <t>038110</t>
         </is>
       </c>
     </row>
@@ -2353,7 +2353,7 @@
         <v>-0.28</v>
       </c>
       <c r="E32" t="n">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="F32" t="n">
         <v>0.74</v>
@@ -2414,7 +2414,7 @@
         <v>0.04</v>
       </c>
       <c r="E33" t="n">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="F33" t="n">
         <v>35.07</v>
@@ -2475,7 +2475,7 @@
         <v>0.72</v>
       </c>
       <c r="E34" t="n">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="F34" t="n">
         <v>8.98</v>
@@ -2536,7 +2536,7 @@
         <v>-0.37</v>
       </c>
       <c r="E35" t="n">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="F35" t="n">
         <v>12.66</v>
@@ -2658,7 +2658,7 @@
         <v>0.42</v>
       </c>
       <c r="E37" t="n">
-        <v>470</v>
+        <v>475</v>
       </c>
       <c r="F37" t="n">
         <v>6.41</v>
@@ -2719,7 +2719,7 @@
         <v>0.16</v>
       </c>
       <c r="E38" t="n">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F38" t="n">
         <v>44.93</v>
@@ -2780,7 +2780,7 @@
         <v>0.74</v>
       </c>
       <c r="E39" t="n">
-        <v>467</v>
+        <v>471</v>
       </c>
       <c r="F39" t="n">
         <v>0.79</v>
@@ -2841,7 +2841,7 @@
         <v>-2.41</v>
       </c>
       <c r="E40" t="n">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="F40" t="n">
         <v>3.74</v>
@@ -2902,7 +2902,7 @@
         <v>0.06</v>
       </c>
       <c r="E41" t="n">
-        <v>618</v>
+        <v>623</v>
       </c>
       <c r="F41" t="n">
         <v>4.74</v>

</xml_diff>

<commit_message>
V8.9.9.5: Final Fix for Research Data and Sidebar Layout
</commit_message>
<xml_diff>
--- a/data/trending_integrated.xlsx
+++ b/data/trending_integrated.xlsx
@@ -523,7 +523,7 @@
         <v>-3.53</v>
       </c>
       <c r="E2" t="n">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F2" t="n">
         <v>2.95</v>
@@ -584,7 +584,7 @@
         <v>-0.28</v>
       </c>
       <c r="E3" t="n">
-        <v>309</v>
+        <v>318</v>
       </c>
       <c r="F3" t="n">
         <v>18.2</v>
@@ -645,7 +645,7 @@
         <v>-1.12</v>
       </c>
       <c r="E4" t="n">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="F4" t="n">
         <v>3.71</v>
@@ -706,7 +706,7 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F5" t="n">
         <v>1.92</v>
@@ -767,7 +767,7 @@
         <v>-0.83</v>
       </c>
       <c r="E6" t="n">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F6" t="n">
         <v>7.85</v>
@@ -828,7 +828,7 @@
         <v>-1.21</v>
       </c>
       <c r="E7" t="n">
-        <v>786</v>
+        <v>790</v>
       </c>
       <c r="F7" t="n">
         <v>11.62</v>
@@ -889,7 +889,7 @@
         <v>-0.54</v>
       </c>
       <c r="E8" t="n">
-        <v>572</v>
+        <v>576</v>
       </c>
       <c r="F8" t="n">
         <v>1.37</v>
@@ -950,7 +950,7 @@
         <v>0.74</v>
       </c>
       <c r="E9" t="n">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="F9" t="n">
         <v>1.91</v>
@@ -1011,7 +1011,7 @@
         <v>1.11</v>
       </c>
       <c r="E10" t="n">
-        <v>1017</v>
+        <v>1072</v>
       </c>
       <c r="F10" t="n">
         <v>1.22</v>
@@ -1072,7 +1072,7 @@
         <v>0.45</v>
       </c>
       <c r="E11" t="n">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="F11" t="n">
         <v>19.75</v>
@@ -1194,7 +1194,7 @@
         <v>0.11</v>
       </c>
       <c r="E13" t="n">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="F13" t="n">
         <v>16.74</v>
@@ -1255,7 +1255,7 @@
         <v>0.19</v>
       </c>
       <c r="E14" t="n">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="F14" t="n">
         <v>45.38</v>
@@ -1377,7 +1377,7 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="E16" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F16" t="n">
         <v>1.8</v>
@@ -1438,7 +1438,7 @@
         <v>-0.14</v>
       </c>
       <c r="E17" t="n">
-        <v>768</v>
+        <v>765</v>
       </c>
       <c r="F17" t="n">
         <v>45.1</v>
@@ -1499,7 +1499,7 @@
         <v>0.41</v>
       </c>
       <c r="E18" t="n">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F18" t="n">
         <v>2.92</v>
@@ -1621,7 +1621,7 @@
         <v>0.08</v>
       </c>
       <c r="E20" t="n">
-        <v>1029</v>
+        <v>1096</v>
       </c>
       <c r="F20" t="n">
         <v>52.69</v>
@@ -1682,7 +1682,7 @@
         <v>0.17</v>
       </c>
       <c r="E21" t="n">
-        <v>451</v>
+        <v>458</v>
       </c>
       <c r="F21" t="n">
         <v>9.01</v>
@@ -1743,7 +1743,7 @@
         <v>-0.7</v>
       </c>
       <c r="E22" t="n">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="F22" t="n">
         <v>1.9</v>
@@ -1804,7 +1804,7 @@
         <v>-0.05</v>
       </c>
       <c r="E23" t="n">
-        <v>1189</v>
+        <v>1521</v>
       </c>
       <c r="F23" t="n">
         <v>48.39</v>
@@ -1926,7 +1926,7 @@
         <v>-0.93</v>
       </c>
       <c r="E25" t="n">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F25" t="n">
         <v>1.35</v>
@@ -2048,7 +2048,7 @@
         <v>-0.34</v>
       </c>
       <c r="E27" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F27" t="n">
         <v>1.53</v>
@@ -2109,7 +2109,7 @@
         <v>-0.08</v>
       </c>
       <c r="E28" t="n">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="F28" t="n">
         <v>9.550000000000001</v>
@@ -2170,7 +2170,7 @@
         <v>0.18</v>
       </c>
       <c r="E29" t="n">
-        <v>804</v>
+        <v>832</v>
       </c>
       <c r="F29" t="n">
         <v>1.54</v>
@@ -2231,7 +2231,7 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="E30" t="n">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F30" t="n">
         <v>7.18</v>
@@ -2353,7 +2353,7 @@
         <v>-0.28</v>
       </c>
       <c r="E32" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F32" t="n">
         <v>0.74</v>
@@ -2414,7 +2414,7 @@
         <v>0.04</v>
       </c>
       <c r="E33" t="n">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="F33" t="n">
         <v>35.07</v>
@@ -2475,7 +2475,7 @@
         <v>0.72</v>
       </c>
       <c r="E34" t="n">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="F34" t="n">
         <v>8.98</v>
@@ -2536,7 +2536,7 @@
         <v>-0.37</v>
       </c>
       <c r="E35" t="n">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="F35" t="n">
         <v>12.66</v>
@@ -2597,7 +2597,7 @@
         <v>0.61</v>
       </c>
       <c r="E36" t="n">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="F36" t="n">
         <v>9.09</v>
@@ -2658,7 +2658,7 @@
         <v>0.42</v>
       </c>
       <c r="E37" t="n">
-        <v>475</v>
+        <v>490</v>
       </c>
       <c r="F37" t="n">
         <v>6.41</v>
@@ -2719,7 +2719,7 @@
         <v>0.16</v>
       </c>
       <c r="E38" t="n">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="F38" t="n">
         <v>44.93</v>
@@ -2780,7 +2780,7 @@
         <v>0.74</v>
       </c>
       <c r="E39" t="n">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="F39" t="n">
         <v>0.79</v>
@@ -2841,7 +2841,7 @@
         <v>-2.41</v>
       </c>
       <c r="E40" t="n">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="F40" t="n">
         <v>3.74</v>
@@ -2902,7 +2902,7 @@
         <v>0.06</v>
       </c>
       <c r="E41" t="n">
-        <v>623</v>
+        <v>630</v>
       </c>
       <c r="F41" t="n">
         <v>4.74</v>

</xml_diff>